<commit_message>
docs: update task status for T34-T36 and T40-T43 in assignment sheet
</commit_message>
<xml_diff>
--- a/Document/phan_cong_do_an_tu_hoc_tieng_anh (1).xlsx
+++ b/Document/phan_cong_do_an_tu_hoc_tieng_anh (1).xlsx
@@ -2856,7 +2856,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K37" t="inlineStr"/>
@@ -2907,7 +2907,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K38" t="inlineStr"/>
@@ -2958,7 +2958,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K39" t="inlineStr"/>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K43" t="inlineStr"/>
@@ -3225,7 +3225,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K44" t="inlineStr"/>
@@ -3276,7 +3276,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K45" t="inlineStr"/>
@@ -3327,7 +3327,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K46" t="inlineStr"/>

</xml_diff>